<commit_message>
add checks on Current Portfolio
</commit_message>
<xml_diff>
--- a/data/asset_classes_constrained_with_curr_weights.xlsx
+++ b/data/asset_classes_constrained_with_curr_weights.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6113f60f932799a7/1Evan/.eff_fron_spyder/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2DF92385-66CB-4D22-B59E-DE21EECDFDC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{2DF92385-66CB-4D22-B59E-DE21EECDFDC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{811F3F70-1321-41F0-9DD8-E01C58784001}"/>
   <bookViews>
-    <workbookView xWindow="40" yWindow="0" windowWidth="25560" windowHeight="13660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Investments" sheetId="1" r:id="rId1"/>
@@ -500,7 +500,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="2">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="D3" s="6">
         <f>0.1/4</f>
@@ -515,7 +515,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="2">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="D4" s="6">
         <f t="shared" ref="D4:D6" si="0">0.1/4</f>
@@ -530,7 +530,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="2">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="D5" s="6">
         <f t="shared" si="0"/>
@@ -545,7 +545,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="2">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="D6" s="6">
         <f t="shared" si="0"/>

</xml_diff>